<commit_message>
2023-4-18 Worked on fig1 and fig2 for WCE meeting
</commit_message>
<xml_diff>
--- a/data/2023-01-25 LA Summary MH v2.xlsx
+++ b/data/2023-01-25 LA Summary MH v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HaroM\Box\Lawrenson Lab\Endometriosis\Rstudio_analysis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE8A54CF-E37A-4C76-8491-8D5FD5A6B95F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{659BBE4F-E1A7-4875-920B-CD883DEFDBA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8025" yWindow="1920" windowWidth="27855" windowHeight="13815" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6060" yWindow="2775" windowWidth="27720" windowHeight="13620" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proportion summary" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1551" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1557" uniqueCount="284">
   <si>
     <t>Patient</t>
   </si>
@@ -1868,6 +1868,7 @@
     <xf numFmtId="0" fontId="11" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="11" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1877,7 +1878,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10878,7 +10878,7 @@
       <c r="I17" s="63">
         <v>1</v>
       </c>
-      <c r="J17" s="225" t="s">
+      <c r="J17" s="226" t="s">
         <v>71</v>
       </c>
       <c r="K17" s="90" t="s">
@@ -10940,7 +10940,7 @@
       <c r="I18" s="63">
         <v>1</v>
       </c>
-      <c r="J18" s="226"/>
+      <c r="J18" s="227"/>
       <c r="K18" s="90" t="s">
         <v>263</v>
       </c>
@@ -11065,7 +11065,7 @@
       <c r="I20" s="63">
         <v>1</v>
       </c>
-      <c r="J20" s="225" t="s">
+      <c r="J20" s="226" t="s">
         <v>73</v>
       </c>
       <c r="K20" s="91" t="s">
@@ -11129,7 +11129,7 @@
       <c r="I21" s="63">
         <v>1</v>
       </c>
-      <c r="J21" s="227"/>
+      <c r="J21" s="228"/>
       <c r="K21" s="91" t="s">
         <v>264</v>
       </c>
@@ -11193,7 +11193,7 @@
       <c r="I22" s="63">
         <v>1</v>
       </c>
-      <c r="J22" s="227"/>
+      <c r="J22" s="228"/>
       <c r="K22" s="91" t="s">
         <v>264</v>
       </c>
@@ -11251,7 +11251,7 @@
       <c r="I23" s="63">
         <v>1</v>
       </c>
-      <c r="J23" s="227"/>
+      <c r="J23" s="228"/>
       <c r="K23" s="91" t="s">
         <v>264</v>
       </c>
@@ -11309,7 +11309,7 @@
       <c r="I24" s="63">
         <v>1</v>
       </c>
-      <c r="J24" s="226"/>
+      <c r="J24" s="227"/>
       <c r="K24" s="92"/>
       <c r="L24" s="35">
         <v>4</v>
@@ -11520,7 +11520,7 @@
       <c r="I27" s="63">
         <v>3</v>
       </c>
-      <c r="J27" s="225" t="s">
+      <c r="J27" s="226" t="s">
         <v>71</v>
       </c>
       <c r="K27" s="90" t="s">
@@ -11588,7 +11588,7 @@
       <c r="I28" s="63">
         <v>3</v>
       </c>
-      <c r="J28" s="226"/>
+      <c r="J28" s="227"/>
       <c r="K28" s="90" t="s">
         <v>263</v>
       </c>
@@ -11780,7 +11780,7 @@
       <c r="I31" s="100">
         <v>5</v>
       </c>
-      <c r="J31" s="225" t="s">
+      <c r="J31" s="226" t="s">
         <v>91</v>
       </c>
       <c r="K31" s="221" t="s">
@@ -11850,7 +11850,7 @@
       <c r="I32" s="63">
         <v>5</v>
       </c>
-      <c r="J32" s="226"/>
+      <c r="J32" s="227"/>
       <c r="K32" s="93" t="s">
         <v>266</v>
       </c>
@@ -11916,7 +11916,7 @@
       <c r="I33" s="63">
         <v>6</v>
       </c>
-      <c r="J33" s="225" t="s">
+      <c r="J33" s="226" t="s">
         <v>99</v>
       </c>
       <c r="K33" s="93" t="s">
@@ -11984,7 +11984,7 @@
       <c r="I34" s="63">
         <v>6</v>
       </c>
-      <c r="J34" s="226"/>
+      <c r="J34" s="227"/>
       <c r="K34" s="93" t="s">
         <v>266</v>
       </c>
@@ -13190,7 +13190,7 @@
       <c r="I53" s="63">
         <v>2</v>
       </c>
-      <c r="J53" s="223" t="s">
+      <c r="J53" s="224" t="s">
         <v>82</v>
       </c>
       <c r="K53" s="109" t="s">
@@ -13252,7 +13252,7 @@
       <c r="I54" s="63">
         <v>2</v>
       </c>
-      <c r="J54" s="224"/>
+      <c r="J54" s="225"/>
       <c r="K54" s="110" t="s">
         <v>265</v>
       </c>
@@ -16425,10 +16425,7 @@
     <row r="106" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H106" s="64"/>
       <c r="I106" s="64"/>
-      <c r="O106" s="228">
-        <f>STDEV(O17:O28,O31:O47,O49:O59,O65:O68,O73:O99,O103:O104)</f>
-        <v>2.876914358347562</v>
-      </c>
+      <c r="O106" s="223"/>
     </row>
     <row r="107" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H107" s="64"/>
@@ -20340,7 +20337,9 @@
       <c r="A7" s="152" t="s">
         <v>189</v>
       </c>
-      <c r="B7" s="51"/>
+      <c r="B7" s="51" t="s">
+        <v>283</v>
+      </c>
       <c r="C7" s="153" t="s">
         <v>74</v>
       </c>
@@ -21632,7 +21631,9 @@
       <c r="A32" s="31" t="s">
         <v>205</v>
       </c>
-      <c r="B32" s="30"/>
+      <c r="B32" s="30" t="s">
+        <v>283</v>
+      </c>
       <c r="C32" s="30" t="s">
         <v>139</v>
       </c>
@@ -21683,7 +21684,9 @@
       <c r="A33" s="31" t="s">
         <v>205</v>
       </c>
-      <c r="B33" s="30"/>
+      <c r="B33" s="30" t="s">
+        <v>283</v>
+      </c>
       <c r="C33" s="30" t="s">
         <v>139</v>
       </c>
@@ -22226,7 +22229,9 @@
       <c r="A43" s="31" t="s">
         <v>218</v>
       </c>
-      <c r="B43" s="30"/>
+      <c r="B43" s="30" t="s">
+        <v>283</v>
+      </c>
       <c r="C43" s="30" t="s">
         <v>172</v>
       </c>
@@ -22273,7 +22278,9 @@
       <c r="A44" s="31" t="s">
         <v>218</v>
       </c>
-      <c r="B44" s="30"/>
+      <c r="B44" s="30" t="s">
+        <v>283</v>
+      </c>
       <c r="C44" s="30" t="s">
         <v>172</v>
       </c>
@@ -22314,7 +22321,9 @@
       <c r="A45" s="38" t="s">
         <v>218</v>
       </c>
-      <c r="B45" s="37"/>
+      <c r="B45" s="37" t="s">
+        <v>283</v>
+      </c>
       <c r="C45" s="37" t="s">
         <v>172</v>
       </c>

</xml_diff>